<commit_message>
Last appendix version before break
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010D7A53-AEF9-0843-B602-262A52D9E1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
+    <workbookView xWindow="38400" yWindow="1860" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
   <sheets>
     <sheet name="constant" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Remove prior for exponent
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/tb_hierarchical/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010D7A53-AEF9-0843-B602-262A52D9E1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D1047F-C745-CC47-8107-DE9F688B139C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="1860" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
+    <workbookView xWindow="39640" yWindow="4000" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
   <sheets>
     <sheet name="constant" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="139">
   <si>
     <t>parameter</t>
   </si>
@@ -1820,15 +1820,6 @@
         <v>131</v>
       </c>
       <c r="B54">
-        <v>0.5</v>
-      </c>
-      <c r="C54" t="s">
-        <v>17</v>
-      </c>
-      <c r="D54">
-        <v>0</v>
-      </c>
-      <c r="E54">
         <v>1</v>
       </c>
       <c r="G54" t="s">

</xml_diff>

<commit_message>
Switch to density-dependent transmission
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/tb_hierarchical/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D1047F-C745-CC47-8107-DE9F688B139C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB61E564-8D77-9246-82AC-BA9A7B51774A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="39640" yWindow="4000" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
@@ -1820,7 +1820,7 @@
         <v>131</v>
       </c>
       <c r="B54">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="G54" t="s">
         <v>132</v>

</xml_diff>

<commit_message>
Revise beta prior for fd model
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/tb_hierarchical/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB61E564-8D77-9246-82AC-BA9A7B51774A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E456ECDB-9F9B-544A-8987-66D4E4D333FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39640" yWindow="4000" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
   <sheets>
     <sheet name="constant" sheetId="1" r:id="rId1"/>
@@ -969,7 +969,7 @@
         <v>14</v>
       </c>
       <c r="B2" s="2">
-        <v>1E-3</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>17</v>
@@ -978,7 +978,7 @@
         <v>1E-4</v>
       </c>
       <c r="E2" s="2">
-        <v>3.0000000000000001E-3</v>
+        <v>1E-3</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>71</v>
@@ -1820,7 +1820,7 @@
         <v>131</v>
       </c>
       <c r="B54">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="G54" t="s">
         <v>132</v>

</xml_diff>

<commit_message>
Stratify by reachability - first steps
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/tb_hierarchical/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010D7A53-AEF9-0843-B602-262A52D9E1D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4721B5E7-D78E-6949-9C06-37AE42E8E0C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="1860" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="141">
   <si>
     <t>parameter</t>
   </si>
@@ -454,6 +454,12 @@
   </si>
   <si>
     <t>Strength of parent-children mixing pattern</t>
+  </si>
+  <si>
+    <t>reachable_pop_frac</t>
+  </si>
+  <si>
+    <t>Proportion of population that is reachable by screening interventions</t>
   </si>
 </sst>
 </file>
@@ -922,7 +928,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57F6C8F8-7718-2F41-B98B-2D455BE12E8B}">
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.5" bestFit="1" customWidth="1"/>
@@ -1833,6 +1839,17 @@
       </c>
       <c r="G54" t="s">
         <v>132</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>139</v>
+      </c>
+      <c r="B55">
+        <v>0.9</v>
+      </c>
+      <c r="G55" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adjust passive detection for unreachable stratum
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/tb_hierarchical/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4721B5E7-D78E-6949-9C06-37AE42E8E0C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94CC3CB9-2871-1841-B1A1-D1797975FDB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="1860" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
+    <workbookView xWindow="38400" yWindow="3240" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
   <sheets>
     <sheet name="constant" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="145">
   <si>
     <t>parameter</t>
   </si>
@@ -460,6 +460,18 @@
   </si>
   <si>
     <t>Proportion of population that is reachable by screening interventions</t>
+  </si>
+  <si>
+    <t>rel_detection_unreachable</t>
+  </si>
+  <si>
+    <t>Relative detection rate of unreachable population under passive case finding (ref. reachable)</t>
+  </si>
+  <si>
+    <t>rel_sus_unreachable</t>
+  </si>
+  <si>
+    <t>Relative susceptibility to infection of unreachable population (ref. reachable)</t>
   </si>
 </sst>
 </file>
@@ -928,7 +940,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57F6C8F8-7718-2F41-B98B-2D455BE12E8B}">
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.5" bestFit="1" customWidth="1"/>
@@ -1850,6 +1862,28 @@
       </c>
       <c r="G55" t="s">
         <v>140</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>141</v>
+      </c>
+      <c r="B56">
+        <v>0</v>
+      </c>
+      <c r="G56" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>143</v>
+      </c>
+      <c r="B57">
+        <v>1.5</v>
+      </c>
+      <c r="G57" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use reachable population for screening-related outputs
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/tb_hierarchical/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94CC3CB9-2871-1841-B1A1-D1797975FDB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB491D1-0E76-2240-9997-DA98C4F4DA2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="3240" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
@@ -1869,7 +1869,7 @@
         <v>141</v>
       </c>
       <c r="B56">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G56" t="s">
         <v>142</v>

</xml_diff>

<commit_message>
Increase prop unreachable to 15%
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/tb_hierarchical/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB491D1-0E76-2240-9997-DA98C4F4DA2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07708E3D-ABBF-A842-A30D-D93B7184B075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="3240" windowWidth="29400" windowHeight="18360" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
   <sheets>
     <sheet name="constant" sheetId="1" r:id="rId1"/>
@@ -1858,7 +1858,7 @@
         <v>139</v>
       </c>
       <c r="B55">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="G55" t="s">
         <v>140</v>

</xml_diff>

<commit_message>
Broaden prior for infectiousness gain rate
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/tb_hierarchical/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E48C201-FCD5-1040-BD10-802C838DD380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CEBC68B-D618-9644-9552-DE3307150337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
@@ -1378,7 +1378,7 @@
         <v>0.5</v>
       </c>
       <c r="E22" s="3">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>88</v>

</xml_diff>

<commit_message>
TST pos now covers all states
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/tb_hierarchical/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CEBC68B-D618-9644-9552-DE3307150337}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E23925FB-7A09-E14E-BA2B-E5A1032ACE26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
@@ -186,15 +186,6 @@
     <t>\tau</t>
   </si>
   <si>
-    <t>prev_se_incipient</t>
-  </si>
-  <si>
-    <t>prev_se_contained</t>
-  </si>
-  <si>
-    <t>prev_se_cleared</t>
-  </si>
-  <si>
     <t>tpt_completion_perc</t>
   </si>
   <si>
@@ -472,6 +463,15 @@
   </si>
   <si>
     <t>Relative susceptibility to infection of unreachable population (ref. reachable)</t>
+  </si>
+  <si>
+    <t>prev_se_incipient_tst</t>
+  </si>
+  <si>
+    <t>prev_se_contained_tst</t>
+  </si>
+  <si>
+    <t>prev_se_cleared_tst</t>
   </si>
 </sst>
 </file>
@@ -999,7 +999,7 @@
         <v>3.0000000000000001E-3</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>27</v>
@@ -1007,7 +1007,7 @@
     </row>
     <row r="3" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B3" s="2">
         <v>0.05</v>
@@ -1022,12 +1022,12 @@
         <v>0.05</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B4" s="2">
         <v>10</v>
@@ -1042,7 +1042,7 @@
         <v>15</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>28</v>
@@ -1050,7 +1050,7 @@
     </row>
     <row r="5" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B5" s="2">
         <v>1.5</v>
@@ -1065,7 +1065,7 @@
         <v>2</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>29</v>
@@ -1088,7 +1088,7 @@
         <v>0.5</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>30</v>
@@ -1111,7 +1111,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>31</v>
@@ -1134,7 +1134,7 @@
         <v>1</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>32</v>
@@ -1148,18 +1148,18 @@
         <v>0.5</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B10" s="4">
         <v>0.4</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>33</v>
@@ -1167,13 +1167,13 @@
     </row>
     <row r="11" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B11" s="5">
         <v>2.4</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>34</v>
@@ -1184,13 +1184,13 @@
     </row>
     <row r="12" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B12" s="5">
         <v>2</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>25</v>
@@ -1198,13 +1198,13 @@
     </row>
     <row r="13" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B13" s="5">
         <v>0.1</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>25</v>
@@ -1212,13 +1212,13 @@
     </row>
     <row r="14" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B14" s="5">
         <v>0.5</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>25</v>
@@ -1226,13 +1226,13 @@
     </row>
     <row r="15" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B15" s="5">
         <v>4.4000000000000004</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>35</v>
@@ -1243,13 +1243,13 @@
     </row>
     <row r="16" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B16" s="5">
         <v>4.4000000000000004</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>25</v>
@@ -1257,13 +1257,13 @@
     </row>
     <row r="17" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B17" s="5">
         <v>2</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>25</v>
@@ -1286,7 +1286,7 @@
         <v>1</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>36</v>
@@ -1312,7 +1312,7 @@
         <v>0.1</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>39</v>
@@ -1338,7 +1338,7 @@
         <v>5</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>40</v>
@@ -1355,7 +1355,7 @@
         <v>1</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>41</v>
@@ -1381,7 +1381,7 @@
         <v>10</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>42</v>
@@ -1398,7 +1398,7 @@
         <v>1</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>43</v>
@@ -1415,7 +1415,7 @@
         <v>0.38900000000000001</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>38</v>
@@ -1426,16 +1426,16 @@
     </row>
     <row r="25" spans="1:9" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B25" s="6">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="I25" s="6" t="s">
         <v>25</v>
@@ -1449,7 +1449,7 @@
         <v>0.4</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>37</v>
@@ -1475,7 +1475,7 @@
         <v>5</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>25</v>
@@ -1489,7 +1489,7 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>48</v>
@@ -1506,7 +1506,7 @@
         <v>40</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>44</v>
@@ -1514,29 +1514,29 @@
     </row>
     <row r="30" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>49</v>
+        <v>142</v>
       </c>
       <c r="B30" s="5">
         <v>0.75</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="31" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>50</v>
+        <v>143</v>
       </c>
       <c r="B31" s="5">
         <v>0.75</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>51</v>
+        <v>144</v>
       </c>
       <c r="B32" s="5">
         <v>0.35</v>
@@ -1551,100 +1551,100 @@
         <v>0.5</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="9" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B33" s="9">
         <v>1</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="9" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B34" s="9">
         <v>1</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="35" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="9" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B35" s="9">
         <v>1</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="36" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="9" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B36" s="9">
         <v>1</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="37" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="10" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B37" s="10">
         <v>0.3</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="10" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B38" s="10">
         <v>1</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="39" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="10" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B39" s="10">
         <v>0.5</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="40" spans="1:7" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="10" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B40" s="10">
         <v>1</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="41" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B41" s="11">
         <v>0.25</v>
@@ -1659,23 +1659,23 @@
         <v>0.52</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B42" s="11">
         <v>1</v>
       </c>
       <c r="G42" s="11" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="43" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="11" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B43" s="11">
         <v>0.85</v>
@@ -1690,73 +1690,73 @@
         <v>0.93</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="44" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="11" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B44" s="11">
         <v>1</v>
       </c>
       <c r="G44" s="11" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="45" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="12" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B45" s="12">
         <v>0</v>
       </c>
       <c r="G45" s="12" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="46" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="12" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B46" s="12">
         <v>1</v>
       </c>
       <c r="G46" s="12" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="47" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="12" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B47" s="12">
         <v>0</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="48" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="12" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B48" s="12">
         <v>1</v>
       </c>
       <c r="G48" s="12" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="49" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="8" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B49" s="8">
         <v>70</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I49" s="8" t="s">
         <v>44</v>
@@ -1770,12 +1770,12 @@
         <v>0</v>
       </c>
       <c r="G50" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B51" s="13">
         <v>2000</v>
@@ -1790,12 +1790,12 @@
         <v>2020</v>
       </c>
       <c r="G51" s="13" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B52" s="13">
         <v>0.1</v>
@@ -1810,12 +1810,12 @@
         <v>0.2</v>
       </c>
       <c r="G52" s="13" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B53">
         <v>0.75</v>
@@ -1830,12 +1830,12 @@
         <v>1</v>
       </c>
       <c r="G53" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B54">
         <v>0.5</v>
@@ -1850,40 +1850,40 @@
         <v>1</v>
       </c>
       <c r="G54" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B55">
         <v>0.85</v>
       </c>
       <c r="G55" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B56">
         <v>0.5</v>
       </c>
       <c r="G56" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B57">
         <v>1.5</v>
       </c>
       <c r="G57" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Remove mixing matrix" commit
</commit_message>
<xml_diff>
--- a/data/parameters.xlsx
+++ b/data/parameters.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rrag0004/Documents/Code/tb_hierarchical/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BED7ACAA-91E3-9044-BCF4-262DC8109B9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E23925FB-7A09-E14E-BA2B-E5A1032ACE26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{D0791FB0-CE82-4F48-97F1-167D990A1A74}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="145">
   <si>
     <t>parameter</t>
   </si>
@@ -438,6 +438,15 @@
     <t>bg_mixing</t>
   </si>
   <si>
+    <t>Background age-agnostic mixing level</t>
+  </si>
+  <si>
+    <t>Spread of assortative mixing pattern (smaller value means more assortativity)</t>
+  </si>
+  <si>
+    <t>Strength of parent-children mixing pattern</t>
+  </si>
+  <si>
     <t>reachable_pop_frac</t>
   </si>
   <si>
@@ -463,15 +472,6 @@
   </si>
   <si>
     <t>prev_se_cleared_tst</t>
-  </si>
-  <si>
-    <t>Background age-agnostic mixing level (0.01 - 0.05)</t>
-  </si>
-  <si>
-    <t>Spread of assortative mixing pattern (smaller value means more assortativity) (5 - 15)</t>
-  </si>
-  <si>
-    <t>Strength of parent-children mixing pattern. (0.1 - 2)</t>
   </si>
 </sst>
 </file>
@@ -1012,8 +1012,17 @@
       <c r="B3" s="2">
         <v>0.05</v>
       </c>
+      <c r="C3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.01</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0.05</v>
+      </c>
       <c r="G3" s="2" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.2">
@@ -1023,8 +1032,17 @@
       <c r="B4" s="2">
         <v>10</v>
       </c>
+      <c r="C4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="2">
+        <v>5</v>
+      </c>
+      <c r="E4" s="2">
+        <v>15</v>
+      </c>
       <c r="G4" s="2" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>28</v>
@@ -1037,8 +1055,17 @@
       <c r="B5" s="2">
         <v>1.5</v>
       </c>
+      <c r="C5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="E5" s="2">
+        <v>2</v>
+      </c>
       <c r="G5" s="2" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>29</v>
@@ -1487,7 +1514,7 @@
     </row>
     <row r="30" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B30" s="5">
         <v>0.75</v>
@@ -1498,7 +1525,7 @@
     </row>
     <row r="31" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B31" s="5">
         <v>0.75</v>
@@ -1509,7 +1536,7 @@
     </row>
     <row r="32" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B32" s="5">
         <v>0.35</v>
@@ -1828,35 +1855,35 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B55">
         <v>0.85</v>
       </c>
       <c r="G55" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B56">
         <v>0.5</v>
       </c>
       <c r="G56" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B57">
         <v>1.5</v>
       </c>
       <c r="G57" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>